<commit_message>
Update intercity pipeline results
</commit_message>
<xml_diff>
--- a/Data/Results/Cleaned/10-07-2026/madhuravoyal_to_silkboard_ev_INTERCITY.xlsx
+++ b/Data/Results/Cleaned/10-07-2026/madhuravoyal_to_silkboard_ev_INTERCITY.xlsx
@@ -25,13 +25,16 @@
     <numFmt numFmtId="167" formatCode="0.000000"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -51,7 +54,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,13 +62,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">

</xml_diff>